<commit_message>
Fix bootstrap data for S2
</commit_message>
<xml_diff>
--- a/scripts/bootstrap/measurement_data/starvation_responses.xlsx
+++ b/scripts/bootstrap/measurement_data/starvation_responses.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>μGrowthDB</author>
   </authors>
@@ -38,6 +38,27 @@
           <t xml:space="preserve">Unique names of individual samples: a bottle, a well in a well-plate, or a mini-bioreactor.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -50,6 +71,27 @@
           <t xml:space="preserve">A compartment within the vessel where growth is measured.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -62,6 +104,27 @@
           <t xml:space="preserve">Measurement time-points in hours (h).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -74,6 +137,27 @@
           <t xml:space="preserve">Optical density values per time-point, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
@@ -86,13 +170,34 @@
           <t xml:space="preserve">pH values per time-point, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>μGrowthDB</author>
   </authors>
@@ -108,6 +213,27 @@
           <t xml:space="preserve">Unique names of individual samples: a bottle, a well in a well-plate, or a mini-bioreactor.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -120,6 +246,27 @@
           <t xml:space="preserve">A compartment within the vessel where growth is measured.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -132,6 +279,27 @@
           <t xml:space="preserve">Measurement time-points in hours (h).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -144,6 +312,27 @@
           <t xml:space="preserve">FC counts values per time-point for strain Roseburia intestinalis L1-82 in Cells/μL, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-36</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>3</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
@@ -156,13 +345,34 @@
           <t xml:space="preserve">FC counts values per time-point for strain Bacteroides thetaiotaomicron VPI-5482 in Cells/μL, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>36</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>13</xdr:colOff>
+                <xdr:row>10</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>μGrowthDB</author>
   </authors>
@@ -178,6 +388,27 @@
           <t xml:space="preserve">Unique names of individual samples: a bottle, a well in a well-plate, or a mini-bioreactor.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -190,6 +421,27 @@
           <t xml:space="preserve">A compartment within the vessel where growth is measured.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -202,6 +454,27 @@
           <t xml:space="preserve">Measurement time-points in hours (h).</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -214,6 +487,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite pyruvate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
@@ -226,6 +520,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite formate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>9</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-3</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
@@ -238,6 +553,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite n-acetylneuraminic acid in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
@@ -250,6 +586,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite glucose in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="H1" authorId="0">
       <text>
@@ -262,6 +619,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite butyrate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="I1" authorId="0">
       <text>
@@ -274,6 +652,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite lactate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="J1" authorId="0">
       <text>
@@ -286,6 +685,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite succinate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="K1" authorId="0">
       <text>
@@ -298,6 +718,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite trehalose in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="L1" authorId="0">
       <text>
@@ -310,6 +751,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite galactose in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="M1" authorId="0">
       <text>
@@ -322,6 +784,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite acetate in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>-12</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="N1" authorId="0">
       <text>
@@ -334,6 +817,27 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite fucose in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>52</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="O1" authorId="0">
       <text>
@@ -346,13 +850,34 @@
           <t xml:space="preserve">Concentration values per time-point for metabolite mannose in mM, use a period (.) as the decimal separator</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>110</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>8</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="567">
   <si>
     <t xml:space="preserve">Biological Replicate</t>
   </si>
@@ -1954,45 +2479,6 @@
   </si>
   <si>
     <t xml:space="preserve">28344676</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10730</t>
-  </si>
-  <si>
-    <t xml:space="preserve">471580</t>
-  </si>
-  <si>
-    <t xml:space="preserve">616425</t>
-  </si>
-  <si>
-    <t xml:space="preserve">829745</t>
-  </si>
-  <si>
-    <t xml:space="preserve">652780</t>
-  </si>
-  <si>
-    <t xml:space="preserve">706755</t>
-  </si>
-  <si>
-    <t xml:space="preserve">463840</t>
-  </si>
-  <si>
-    <t xml:space="preserve">592370</t>
-  </si>
-  <si>
-    <t xml:space="preserve">469770</t>
-  </si>
-  <si>
-    <t xml:space="preserve">671170</t>
-  </si>
-  <si>
-    <t xml:space="preserve">541885</t>
-  </si>
-  <si>
-    <t xml:space="preserve">708485</t>
   </si>
   <si>
     <t xml:space="preserve">33313</t>
@@ -2315,34 +2801,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -12607,9 +13093,7 @@
       <c r="D242" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="E242" s="6" t="n">
-        <v>951</v>
-      </c>
+      <c r="E242" s="6"/>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="3" t="s">
@@ -12624,9 +13108,7 @@
       <c r="D243" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="E243" s="6" t="n">
-        <v>10412</v>
-      </c>
+      <c r="E243" s="6"/>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="3" t="s">
@@ -12639,9 +13121,7 @@
         <v>8</v>
       </c>
       <c r="D244" s="6"/>
-      <c r="E244" s="6" t="n">
-        <v>596610</v>
-      </c>
+      <c r="E244" s="6"/>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="3" t="s">
@@ -12656,9 +13136,7 @@
       <c r="D245" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E245" s="6" t="n">
-        <v>461520</v>
-      </c>
+      <c r="E245" s="6"/>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="3" t="s">
@@ -12673,9 +13151,7 @@
       <c r="D246" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E246" s="6" t="n">
-        <v>312390</v>
-      </c>
+      <c r="E246" s="6"/>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="3" t="s">
@@ -15587,7 +16063,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8"/>
@@ -23064,28 +23540,26 @@
       <c r="D256" s="6" t="n">
         <v>9.66</v>
       </c>
-      <c r="E256" s="6" t="n">
-        <v>1.71</v>
+      <c r="E256" s="0" t="n">
+        <v>0.88</v>
       </c>
       <c r="F256" s="6"/>
       <c r="G256" s="6" t="n">
         <v>7.38</v>
       </c>
-      <c r="H256" s="6" t="s">
-        <v>534</v>
-      </c>
-      <c r="I256" s="6" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="J256" s="6" t="n">
+      <c r="H256" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I256" s="0" t="n">
         <v>0.39</v>
       </c>
-      <c r="K256" s="6" t="n">
-        <v>0</v>
+      <c r="J256" s="6"/>
+      <c r="K256" s="0" t="n">
+        <v>0.65</v>
       </c>
       <c r="L256" s="6"/>
-      <c r="M256" s="6" t="n">
-        <v>0.65</v>
+      <c r="M256" s="0" t="n">
+        <v>1.71</v>
       </c>
       <c r="N256" s="6"/>
       <c r="O256" s="6"/>
@@ -23103,28 +23577,26 @@
       <c r="D257" s="6" t="n">
         <v>9.52</v>
       </c>
-      <c r="E257" s="6" t="n">
-        <v>1.86</v>
+      <c r="E257" s="0" t="n">
+        <v>0.89</v>
       </c>
       <c r="F257" s="6"/>
       <c r="G257" s="6" t="n">
         <v>7.24</v>
       </c>
-      <c r="H257" s="6" t="s">
-        <v>535</v>
-      </c>
-      <c r="I257" s="6" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="J257" s="6" t="n">
+      <c r="H257" s="0" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I257" s="0" t="n">
         <v>0.37</v>
       </c>
-      <c r="K257" s="6" t="n">
-        <v>0.04</v>
+      <c r="J257" s="6"/>
+      <c r="K257" s="0" t="n">
+        <v>0.64</v>
       </c>
       <c r="L257" s="6"/>
-      <c r="M257" s="6" t="n">
-        <v>0.64</v>
+      <c r="M257" s="0" t="n">
+        <v>1.88</v>
       </c>
       <c r="N257" s="6"/>
       <c r="O257" s="6"/>
@@ -23142,26 +23614,26 @@
       <c r="D258" s="6" t="n">
         <v>9.63</v>
       </c>
-      <c r="E258" s="6" t="n">
-        <v>3.09</v>
+      <c r="E258" s="0" t="n">
+        <v>0.88</v>
       </c>
       <c r="F258" s="6"/>
       <c r="G258" s="6" t="n">
         <v>6.19</v>
       </c>
-      <c r="H258" s="6"/>
-      <c r="I258" s="6" t="n">
+      <c r="H258" s="0" t="n">
         <v>0.88</v>
       </c>
-      <c r="J258" s="6" t="n">
+      <c r="I258" s="0" t="n">
         <v>0.63</v>
       </c>
-      <c r="K258" s="6" t="n">
-        <v>0.88</v>
+      <c r="J258" s="6"/>
+      <c r="K258" s="0" t="n">
+        <v>0.63</v>
       </c>
       <c r="L258" s="6"/>
-      <c r="M258" s="6" t="n">
-        <v>0.63</v>
+      <c r="M258" s="0" t="n">
+        <v>2.84</v>
       </c>
       <c r="N258" s="6"/>
       <c r="O258" s="6"/>
@@ -23179,28 +23651,26 @@
       <c r="D259" s="6" t="n">
         <v>8.64</v>
       </c>
-      <c r="E259" s="6" t="n">
-        <v>5.41</v>
+      <c r="E259" s="0" t="n">
+        <v>0.82</v>
       </c>
       <c r="F259" s="6"/>
       <c r="G259" s="6" t="n">
         <v>1.89</v>
       </c>
-      <c r="H259" s="6" t="s">
-        <v>536</v>
-      </c>
-      <c r="I259" s="6" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="J259" s="6" t="n">
+      <c r="H259" s="0" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="I259" s="0" t="n">
         <v>1.32</v>
       </c>
-      <c r="K259" s="6" t="n">
-        <v>3.81</v>
+      <c r="J259" s="6"/>
+      <c r="K259" s="0" t="n">
+        <v>0.61</v>
       </c>
       <c r="L259" s="6"/>
-      <c r="M259" s="6" t="n">
-        <v>0.61</v>
+      <c r="M259" s="0" t="n">
+        <v>5.06</v>
       </c>
       <c r="N259" s="6"/>
       <c r="O259" s="6"/>
@@ -23218,28 +23688,26 @@
       <c r="D260" s="6" t="n">
         <v>1.12</v>
       </c>
-      <c r="E260" s="6" t="n">
-        <v>6.34</v>
+      <c r="E260" s="0" t="n">
+        <v>0.98</v>
       </c>
       <c r="F260" s="6"/>
       <c r="G260" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="H260" s="6" t="s">
-        <v>537</v>
-      </c>
-      <c r="I260" s="6" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J260" s="6" t="n">
+      <c r="H260" s="0" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="I260" s="0" t="n">
         <v>2.39</v>
       </c>
-      <c r="K260" s="6" t="n">
-        <v>8.15</v>
+      <c r="J260" s="6"/>
+      <c r="K260" s="0" t="n">
+        <v>0.58</v>
       </c>
       <c r="L260" s="6"/>
-      <c r="M260" s="6" t="n">
-        <v>0.58</v>
+      <c r="M260" s="0" t="n">
+        <v>5.97</v>
       </c>
       <c r="N260" s="6"/>
       <c r="O260" s="6"/>
@@ -23257,28 +23725,26 @@
       <c r="D261" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="E261" s="6" t="n">
-        <v>6.33</v>
+      <c r="E261" s="0" t="n">
+        <v>1.11</v>
       </c>
       <c r="F261" s="6"/>
       <c r="G261" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="H261" s="6" t="s">
-        <v>538</v>
-      </c>
-      <c r="I261" s="6" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="J261" s="6" t="n">
+      <c r="H261" s="0" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="I261" s="0" t="n">
         <v>2.19</v>
       </c>
-      <c r="K261" s="6" t="n">
-        <v>9.1</v>
+      <c r="J261" s="6"/>
+      <c r="K261" s="0" t="n">
+        <v>0.57</v>
       </c>
       <c r="L261" s="6"/>
-      <c r="M261" s="6" t="n">
-        <v>0.57</v>
+      <c r="M261" s="0" t="n">
+        <v>6.19</v>
       </c>
       <c r="N261" s="6"/>
       <c r="O261" s="6"/>
@@ -23296,28 +23762,26 @@
       <c r="D262" s="6" t="n">
         <v>0.08</v>
       </c>
-      <c r="E262" s="6" t="n">
-        <v>6.74</v>
+      <c r="E262" s="0" t="n">
+        <v>0.98</v>
       </c>
       <c r="F262" s="6"/>
       <c r="G262" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="H262" s="6" t="s">
-        <v>539</v>
-      </c>
-      <c r="I262" s="6" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J262" s="6" t="n">
+      <c r="H262" s="0" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="I262" s="0" t="n">
         <v>2.02</v>
       </c>
-      <c r="K262" s="6" t="n">
-        <v>9.08</v>
+      <c r="J262" s="6"/>
+      <c r="K262" s="0" t="n">
+        <v>0.55</v>
       </c>
       <c r="L262" s="6"/>
-      <c r="M262" s="6" t="n">
-        <v>0.55</v>
+      <c r="M262" s="0" t="n">
+        <v>6.42</v>
       </c>
       <c r="N262" s="6"/>
       <c r="O262" s="6"/>
@@ -23335,28 +23799,26 @@
       <c r="D263" s="6" t="n">
         <v>0.07</v>
       </c>
-      <c r="E263" s="6" t="n">
-        <v>6.95</v>
+      <c r="E263" s="0" t="n">
+        <v>0.91</v>
       </c>
       <c r="F263" s="6"/>
       <c r="G263" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="H263" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="I263" s="6" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="J263" s="6" t="n">
+      <c r="H263" s="0" t="n">
+        <v>9.55</v>
+      </c>
+      <c r="I263" s="0" t="n">
         <v>1.5</v>
       </c>
-      <c r="K263" s="6" t="n">
-        <v>9.55</v>
+      <c r="J263" s="6"/>
+      <c r="K263" s="0" t="n">
+        <v>0.54</v>
       </c>
       <c r="L263" s="6"/>
-      <c r="M263" s="6" t="n">
-        <v>0.54</v>
+      <c r="M263" s="0" t="n">
+        <v>5.89</v>
       </c>
       <c r="N263" s="6"/>
       <c r="O263" s="6"/>
@@ -23374,28 +23836,26 @@
       <c r="D264" s="6" t="n">
         <v>0.13</v>
       </c>
-      <c r="E264" s="6" t="n">
-        <v>6.8</v>
+      <c r="E264" s="0" t="n">
+        <v>1.14</v>
       </c>
       <c r="F264" s="6"/>
       <c r="G264" s="6" t="n">
         <v>0.24</v>
       </c>
-      <c r="H264" s="6" t="s">
-        <v>541</v>
-      </c>
-      <c r="I264" s="6" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="J264" s="6" t="n">
+      <c r="H264" s="0" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="I264" s="0" t="n">
         <v>1.05</v>
       </c>
-      <c r="K264" s="6" t="n">
-        <v>9.4</v>
+      <c r="J264" s="6"/>
+      <c r="K264" s="0" t="n">
+        <v>0.63</v>
       </c>
       <c r="L264" s="6"/>
-      <c r="M264" s="6" t="n">
-        <v>0.63</v>
+      <c r="M264" s="0" t="n">
+        <v>6.7</v>
       </c>
       <c r="N264" s="6"/>
       <c r="O264" s="6"/>
@@ -23413,28 +23873,26 @@
       <c r="D265" s="6" t="n">
         <v>0.13</v>
       </c>
-      <c r="E265" s="6" t="n">
-        <v>6.78</v>
+      <c r="E265" s="0" t="n">
+        <v>1.14</v>
       </c>
       <c r="F265" s="6"/>
       <c r="G265" s="6" t="n">
         <v>0.23</v>
       </c>
-      <c r="H265" s="6" t="s">
-        <v>542</v>
-      </c>
-      <c r="I265" s="6" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="J265" s="6" t="n">
+      <c r="H265" s="0" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="I265" s="0" t="n">
         <v>0.51</v>
       </c>
-      <c r="K265" s="6" t="n">
-        <v>9.66</v>
+      <c r="J265" s="6"/>
+      <c r="K265" s="0" t="n">
+        <v>0.59</v>
       </c>
       <c r="L265" s="6"/>
-      <c r="M265" s="6" t="n">
-        <v>0.59</v>
+      <c r="M265" s="0" t="n">
+        <v>6.67</v>
       </c>
       <c r="N265" s="6"/>
       <c r="O265" s="6"/>
@@ -23452,28 +23910,26 @@
       <c r="D266" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E266" s="6" t="n">
-        <v>6.54</v>
+      <c r="E266" s="0" t="n">
+        <v>1.17</v>
       </c>
       <c r="F266" s="6"/>
       <c r="G266" s="6" t="n">
         <v>0.22</v>
       </c>
-      <c r="H266" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="I266" s="6" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="J266" s="6" t="n">
+      <c r="H266" s="0" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="I266" s="0" t="n">
         <v>0.35</v>
       </c>
-      <c r="K266" s="6" t="n">
-        <v>10.02</v>
+      <c r="J266" s="6"/>
+      <c r="K266" s="0" t="n">
+        <v>0.54</v>
       </c>
       <c r="L266" s="6"/>
-      <c r="M266" s="6" t="n">
-        <v>0.54</v>
+      <c r="M266" s="0" t="n">
+        <v>6.52</v>
       </c>
       <c r="N266" s="6"/>
       <c r="O266" s="6"/>
@@ -23491,28 +23947,26 @@
       <c r="D267" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E267" s="6" t="n">
-        <v>6.41</v>
+      <c r="E267" s="0" t="n">
+        <v>1.12</v>
       </c>
       <c r="F267" s="6"/>
       <c r="G267" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H267" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="I267" s="6" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="J267" s="6" t="n">
+      <c r="H267" s="0" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="I267" s="0" t="n">
         <v>0.33</v>
       </c>
-      <c r="K267" s="6" t="n">
-        <v>10.07</v>
+      <c r="J267" s="6"/>
+      <c r="K267" s="0" t="n">
+        <v>0.52</v>
       </c>
       <c r="L267" s="6"/>
-      <c r="M267" s="6" t="n">
-        <v>0.52</v>
+      <c r="M267" s="0" t="n">
+        <v>6.37</v>
       </c>
       <c r="N267" s="6"/>
       <c r="O267" s="6"/>
@@ -23530,28 +23984,26 @@
       <c r="D268" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E268" s="6" t="n">
-        <v>6.14</v>
+      <c r="E268" s="0" t="n">
+        <v>1.16</v>
       </c>
       <c r="F268" s="6"/>
       <c r="G268" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H268" s="6" t="s">
-        <v>545</v>
-      </c>
-      <c r="I268" s="6" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="J268" s="6" t="n">
+      <c r="H268" s="0" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="I268" s="0" t="n">
         <v>0.37</v>
       </c>
-      <c r="K268" s="6" t="n">
-        <v>10.39</v>
+      <c r="J268" s="6"/>
+      <c r="K268" s="0" t="n">
+        <v>0.46</v>
       </c>
       <c r="L268" s="6"/>
-      <c r="M268" s="6" t="n">
-        <v>0.46</v>
+      <c r="M268" s="0" t="n">
+        <v>6.13</v>
       </c>
       <c r="N268" s="6"/>
       <c r="O268" s="6"/>
@@ -23569,28 +24021,26 @@
       <c r="D269" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="E269" s="6" t="n">
-        <v>5.57</v>
+      <c r="E269" s="0" t="n">
+        <v>1.17</v>
       </c>
       <c r="F269" s="6"/>
       <c r="G269" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H269" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="I269" s="6" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="J269" s="6" t="n">
+      <c r="H269" s="0" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="I269" s="0" t="n">
         <v>0.37</v>
       </c>
-      <c r="K269" s="6" t="n">
-        <v>10.55</v>
+      <c r="J269" s="6"/>
+      <c r="K269" s="0" t="n">
+        <v>0.4</v>
       </c>
       <c r="L269" s="6"/>
-      <c r="M269" s="6" t="n">
-        <v>0.4</v>
+      <c r="M269" s="0" t="n">
+        <v>6.01</v>
       </c>
       <c r="N269" s="6"/>
       <c r="O269" s="6"/>
@@ -24154,10 +24604,10 @@
         <v>1.81</v>
       </c>
       <c r="N284" s="6" t="s">
-        <v>547</v>
+        <v>534</v>
       </c>
       <c r="O284" s="6" t="s">
-        <v>548</v>
+        <v>535</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24687,16 +25137,16 @@
         <v>0.7</v>
       </c>
       <c r="L297" s="6" t="s">
-        <v>549</v>
+        <v>536</v>
       </c>
       <c r="M297" s="6" t="n">
         <v>11.38</v>
       </c>
       <c r="N297" s="6" t="s">
-        <v>550</v>
+        <v>537</v>
       </c>
       <c r="O297" s="6" t="s">
-        <v>551</v>
+        <v>538</v>
       </c>
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24734,16 +25184,16 @@
         <v>0.7</v>
       </c>
       <c r="L298" s="6" t="s">
-        <v>552</v>
+        <v>539</v>
       </c>
       <c r="M298" s="6" t="n">
         <v>11.36</v>
       </c>
       <c r="N298" s="6" t="s">
-        <v>553</v>
+        <v>540</v>
       </c>
       <c r="O298" s="6" t="s">
-        <v>554</v>
+        <v>541</v>
       </c>
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24781,16 +25231,16 @@
         <v>0.69</v>
       </c>
       <c r="L299" s="6" t="s">
-        <v>555</v>
+        <v>542</v>
       </c>
       <c r="M299" s="6" t="n">
         <v>11.38</v>
       </c>
       <c r="N299" s="6" t="s">
-        <v>556</v>
+        <v>543</v>
       </c>
       <c r="O299" s="6" t="s">
-        <v>557</v>
+        <v>544</v>
       </c>
     </row>
     <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25202,10 +25652,10 @@
         <v>1.79</v>
       </c>
       <c r="N316" s="6" t="s">
-        <v>558</v>
+        <v>545</v>
       </c>
       <c r="O316" s="6" t="s">
-        <v>559</v>
+        <v>546</v>
       </c>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25735,16 +26185,16 @@
         <v>0.7</v>
       </c>
       <c r="L329" s="6" t="s">
-        <v>560</v>
+        <v>547</v>
       </c>
       <c r="M329" s="6" t="n">
         <v>11.48</v>
       </c>
       <c r="N329" s="6" t="s">
-        <v>561</v>
+        <v>548</v>
       </c>
       <c r="O329" s="6" t="s">
-        <v>562</v>
+        <v>549</v>
       </c>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25782,16 +26232,16 @@
         <v>0.7</v>
       </c>
       <c r="L330" s="6" t="s">
-        <v>563</v>
+        <v>550</v>
       </c>
       <c r="M330" s="6" t="n">
         <v>11.48</v>
       </c>
       <c r="N330" s="6" t="s">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="O330" s="6" t="s">
-        <v>565</v>
+        <v>552</v>
       </c>
     </row>
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25829,16 +26279,16 @@
         <v>0.7</v>
       </c>
       <c r="L331" s="6" t="s">
-        <v>566</v>
+        <v>553</v>
       </c>
       <c r="M331" s="6" t="n">
         <v>11.51</v>
       </c>
       <c r="N331" s="6" t="s">
-        <v>567</v>
+        <v>554</v>
       </c>
       <c r="O331" s="6" t="s">
-        <v>568</v>
+        <v>555</v>
       </c>
     </row>
     <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26250,10 +26700,10 @@
         <v>1.73</v>
       </c>
       <c r="N348" s="6" t="s">
-        <v>569</v>
+        <v>556</v>
       </c>
       <c r="O348" s="6" t="s">
-        <v>570</v>
+        <v>557</v>
       </c>
     </row>
     <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26783,16 +27233,16 @@
         <v>0.7</v>
       </c>
       <c r="L361" s="6" t="s">
-        <v>571</v>
+        <v>558</v>
       </c>
       <c r="M361" s="6" t="n">
         <v>11.23</v>
       </c>
       <c r="N361" s="6" t="s">
-        <v>572</v>
+        <v>559</v>
       </c>
       <c r="O361" s="6" t="s">
-        <v>573</v>
+        <v>560</v>
       </c>
     </row>
     <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26830,16 +27280,16 @@
         <v>0.7</v>
       </c>
       <c r="L362" s="6" t="s">
-        <v>574</v>
+        <v>561</v>
       </c>
       <c r="M362" s="6" t="n">
         <v>11.3</v>
       </c>
       <c r="N362" s="6" t="s">
-        <v>575</v>
+        <v>562</v>
       </c>
       <c r="O362" s="6" t="s">
-        <v>576</v>
+        <v>563</v>
       </c>
     </row>
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26877,16 +27327,16 @@
         <v>0.7</v>
       </c>
       <c r="L363" s="6" t="s">
-        <v>577</v>
+        <v>564</v>
       </c>
       <c r="M363" s="6" t="n">
         <v>11.27</v>
       </c>
       <c r="N363" s="6" t="s">
-        <v>578</v>
+        <v>565</v>
       </c>
       <c r="O363" s="6" t="s">
-        <v>579</v>
+        <v>566</v>
       </c>
     </row>
     <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update S2 bootstrap measurement data
</commit_message>
<xml_diff>
--- a/scripts/bootstrap/measurement_data/starvation_responses.xlsx
+++ b/scripts/bootstrap/measurement_data/starvation_responses.xlsx
@@ -44,13 +44,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -77,13 +77,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -110,13 +110,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -143,13 +143,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -176,13 +176,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -219,13 +219,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -252,13 +252,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -285,13 +285,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>3</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -324,9 +324,9 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-36</xdr:colOff>
+                <xdr:colOff>-21</xdr:colOff>
                 <xdr:row>9</xdr:row>
-                <xdr:rowOff>3</xdr:rowOff>
+                <xdr:rowOff>2</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -351,13 +351,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>36</xdr:colOff>
+                <xdr:colOff>21</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>3</xdr:col>
-                <xdr:colOff>13</xdr:colOff>
+                <xdr:colOff>8</xdr:colOff>
                 <xdr:row>10</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -394,13 +394,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -427,13 +427,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -460,13 +460,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>3</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -493,13 +493,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -526,13 +526,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>9</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-3</xdr:colOff>
+                <xdr:colOff>-2</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -565,7 +565,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -598,7 +598,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -631,7 +631,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -664,7 +664,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -697,7 +697,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -730,7 +730,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -763,7 +763,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -796,9 +796,9 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>-12</xdr:colOff>
+                <xdr:colOff>-7</xdr:colOff>
                 <xdr:row>4</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
+                <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -829,7 +829,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>52</xdr:colOff>
+                <xdr:colOff>30</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -856,13 +856,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>110</xdr:colOff>
+                <xdr:colOff>64</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>8</xdr:colOff>
+                <xdr:colOff>5</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -4443,10 +4443,10 @@
       <c r="C104" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D104" s="3" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="E104" s="3" t="n">
+      <c r="D104" s="0" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="E104" s="0" t="n">
         <v>6.6</v>
       </c>
     </row>
@@ -4460,10 +4460,10 @@
       <c r="C105" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D105" s="3" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="E105" s="3" t="n">
+      <c r="D105" s="0" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="E105" s="0" t="n">
         <v>6.61</v>
       </c>
     </row>
@@ -4477,10 +4477,10 @@
       <c r="C106" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D106" s="3" t="n">
-        <v>0.407</v>
-      </c>
-      <c r="E106" s="3" t="n">
+      <c r="D106" s="0" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="E106" s="0" t="n">
         <v>6.15</v>
       </c>
     </row>
@@ -4494,11 +4494,11 @@
       <c r="C107" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="D107" s="3" t="n">
-        <v>0.795</v>
-      </c>
-      <c r="E107" s="3" t="n">
-        <v>5.42</v>
+      <c r="D107" s="0" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E107" s="0" t="n">
+        <v>5.47</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4511,10 +4511,10 @@
       <c r="C108" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D108" s="3" t="n">
-        <v>0.966</v>
-      </c>
-      <c r="E108" s="3" t="n">
+      <c r="D108" s="0" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="E108" s="0" t="n">
         <v>5.09</v>
       </c>
     </row>
@@ -4528,10 +4528,10 @@
       <c r="C109" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D109" s="3" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="E109" s="3" t="n">
+      <c r="D109" s="0" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="E109" s="0" t="n">
         <v>5.04</v>
       </c>
     </row>
@@ -4545,10 +4545,10 @@
       <c r="C110" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="D110" s="3" t="n">
-        <v>0.661</v>
-      </c>
-      <c r="E110" s="3" t="n">
+      <c r="D110" s="0" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E110" s="0" t="n">
         <v>4.97</v>
       </c>
     </row>
@@ -4562,10 +4562,10 @@
       <c r="C111" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="D111" s="3" t="n">
-        <v>0.657</v>
-      </c>
-      <c r="E111" s="3" t="n">
+      <c r="D111" s="0" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="E111" s="0" t="n">
         <v>4.97</v>
       </c>
     </row>
@@ -4579,10 +4579,10 @@
       <c r="C112" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="D112" s="3" t="n">
-        <v>0.872</v>
-      </c>
-      <c r="E112" s="3" t="n">
+      <c r="D112" s="0" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E112" s="0" t="n">
         <v>5.01</v>
       </c>
     </row>
@@ -4596,11 +4596,11 @@
       <c r="C113" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="D113" s="3" t="n">
-        <v>0.911</v>
-      </c>
-      <c r="E113" s="3" t="n">
-        <v>5.14</v>
+      <c r="D113" s="0" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="E113" s="0" t="n">
+        <v>5.09</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4613,10 +4613,10 @@
       <c r="C114" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D114" s="3" t="n">
-        <v>0.924</v>
-      </c>
-      <c r="E114" s="3" t="n">
+      <c r="D114" s="0" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="E114" s="0" t="n">
         <v>5.09</v>
       </c>
     </row>
@@ -4630,10 +4630,10 @@
       <c r="C115" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="D115" s="3" t="n">
-        <v>0.921</v>
-      </c>
-      <c r="E115" s="3" t="n">
+      <c r="D115" s="0" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="E115" s="0" t="n">
         <v>5.09</v>
       </c>
     </row>
@@ -4647,10 +4647,10 @@
       <c r="C116" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="D116" s="3" t="n">
-        <v>0.911</v>
-      </c>
-      <c r="E116" s="3" t="n">
+      <c r="D116" s="0" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="E116" s="0" t="n">
         <v>5.14</v>
       </c>
     </row>
@@ -4664,11 +4664,11 @@
       <c r="C117" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="D117" s="3" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="E117" s="3" t="n">
-        <v>5.13</v>
+      <c r="D117" s="0" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="E117" s="0" t="n">
+        <v>5.09</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18549,27 +18549,27 @@
       <c r="C104" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D104" s="6" t="n">
-        <v>9.62</v>
-      </c>
-      <c r="E104" s="6" t="n">
-        <v>0.81</v>
+      <c r="D104" s="0" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="E104" s="0" t="n">
+        <v>0.85</v>
       </c>
       <c r="F104" s="6"/>
-      <c r="G104" s="6" t="n">
-        <v>7.42</v>
+      <c r="G104" s="0" t="n">
+        <v>7.5</v>
       </c>
       <c r="H104" s="6"/>
-      <c r="I104" s="6" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="J104" s="6" t="n">
-        <v>0.56</v>
+      <c r="I104" s="0" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J104" s="0" t="n">
+        <v>0.57</v>
       </c>
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
-      <c r="M104" s="6" t="n">
-        <v>1.59</v>
+      <c r="M104" s="0" t="n">
+        <v>1.53</v>
       </c>
       <c r="N104" s="6"/>
       <c r="O104" s="6"/>
@@ -18584,27 +18584,27 @@
       <c r="C105" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D105" s="6" t="n">
-        <v>9.78</v>
-      </c>
-      <c r="E105" s="6" t="n">
-        <v>0.89</v>
+      <c r="D105" s="0" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="E105" s="0" t="n">
+        <v>0.9</v>
       </c>
       <c r="F105" s="6"/>
-      <c r="G105" s="6" t="n">
-        <v>7.48</v>
+      <c r="G105" s="0" t="n">
+        <v>7.29</v>
       </c>
       <c r="H105" s="6"/>
-      <c r="I105" s="6" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="J105" s="6" t="n">
-        <v>0.61</v>
+      <c r="I105" s="0" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J105" s="0" t="n">
+        <v>0.6</v>
       </c>
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
-      <c r="M105" s="6" t="n">
-        <v>1.94</v>
+      <c r="M105" s="0" t="n">
+        <v>1.89</v>
       </c>
       <c r="N105" s="6"/>
       <c r="O105" s="6"/>
@@ -18619,27 +18619,27 @@
       <c r="C106" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D106" s="6" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="E106" s="6" t="n">
-        <v>1.86</v>
+      <c r="D106" s="0" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="E106" s="0" t="n">
+        <v>1.92</v>
       </c>
       <c r="F106" s="6"/>
-      <c r="G106" s="6" t="n">
+      <c r="G106" s="0" t="n">
         <v>5.99</v>
       </c>
       <c r="H106" s="6"/>
-      <c r="I106" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="J106" s="6" t="n">
-        <v>2.15</v>
+      <c r="I106" s="0" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J106" s="0" t="n">
+        <v>2.2</v>
       </c>
       <c r="K106" s="6"/>
       <c r="L106" s="6"/>
-      <c r="M106" s="6" t="n">
-        <v>3.64</v>
+      <c r="M106" s="0" t="n">
+        <v>3.73</v>
       </c>
       <c r="N106" s="6"/>
       <c r="O106" s="6"/>
@@ -18654,27 +18654,27 @@
       <c r="C107" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="D107" s="6" t="n">
-        <v>7.86</v>
-      </c>
-      <c r="E107" s="6" t="n">
-        <v>2.44</v>
+      <c r="D107" s="0" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E107" s="0" t="n">
+        <v>2.46</v>
       </c>
       <c r="F107" s="6"/>
-      <c r="G107" s="6" t="n">
-        <v>3.19</v>
+      <c r="G107" s="0" t="n">
+        <v>3.08</v>
       </c>
       <c r="H107" s="6"/>
-      <c r="I107" s="6" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="J107" s="6" t="n">
-        <v>4.97</v>
+      <c r="I107" s="0" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J107" s="0" t="n">
+        <v>4.98</v>
       </c>
       <c r="K107" s="6"/>
       <c r="L107" s="6"/>
-      <c r="M107" s="6" t="n">
-        <v>6.89</v>
+      <c r="M107" s="0" t="n">
+        <v>7.01</v>
       </c>
       <c r="N107" s="6"/>
       <c r="O107" s="6"/>
@@ -18689,27 +18689,27 @@
       <c r="C108" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D108" s="6" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="E108" s="6" t="n">
-        <v>2.49</v>
+      <c r="D108" s="0" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="E108" s="0" t="n">
+        <v>2.46</v>
       </c>
       <c r="F108" s="6"/>
-      <c r="G108" s="6" t="n">
-        <v>0.73</v>
+      <c r="G108" s="0" t="n">
+        <v>0.64</v>
       </c>
       <c r="H108" s="6"/>
-      <c r="I108" s="6" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="J108" s="6" t="n">
-        <v>7.22</v>
+      <c r="I108" s="0" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="J108" s="0" t="n">
+        <v>7.63</v>
       </c>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
-      <c r="M108" s="6" t="n">
-        <v>10.73</v>
+      <c r="M108" s="0" t="n">
+        <v>10.79</v>
       </c>
       <c r="N108" s="6"/>
       <c r="O108" s="6"/>
@@ -18724,27 +18724,27 @@
       <c r="C109" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D109" s="6" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="E109" s="6" t="n">
-        <v>2.39</v>
+      <c r="D109" s="0" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="E109" s="0" t="n">
+        <v>2.35</v>
       </c>
       <c r="F109" s="6"/>
-      <c r="G109" s="6" t="n">
+      <c r="G109" s="0" t="n">
         <v>0.15</v>
       </c>
       <c r="H109" s="6"/>
-      <c r="I109" s="6" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="J109" s="6" t="n">
-        <v>9.57</v>
+      <c r="I109" s="0" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="J109" s="0" t="n">
+        <v>9.63</v>
       </c>
       <c r="K109" s="6"/>
       <c r="L109" s="6"/>
-      <c r="M109" s="6" t="n">
-        <v>13.24</v>
+      <c r="M109" s="0" t="n">
+        <v>12.75</v>
       </c>
       <c r="N109" s="6"/>
       <c r="O109" s="6"/>
@@ -18759,27 +18759,27 @@
       <c r="C110" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="D110" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E110" s="6" t="n">
-        <v>2.19</v>
+      <c r="D110" s="0" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E110" s="0" t="n">
+        <v>2.25</v>
       </c>
       <c r="F110" s="6"/>
-      <c r="G110" s="6" t="n">
-        <v>0.13</v>
+      <c r="G110" s="0" t="n">
+        <v>0.14</v>
       </c>
       <c r="H110" s="6"/>
-      <c r="I110" s="6" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="J110" s="6" t="n">
-        <v>10.12</v>
+      <c r="I110" s="0" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="J110" s="0" t="n">
+        <v>10.32</v>
       </c>
       <c r="K110" s="6"/>
       <c r="L110" s="6"/>
-      <c r="M110" s="6" t="n">
-        <v>13.21</v>
+      <c r="M110" s="0" t="n">
+        <v>13.01</v>
       </c>
       <c r="N110" s="6"/>
       <c r="O110" s="6"/>
@@ -18794,27 +18794,27 @@
       <c r="C111" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="D111" s="6" t="n">
+      <c r="D111" s="0" t="n">
         <v>0.58</v>
       </c>
-      <c r="E111" s="6" t="n">
-        <v>2.17</v>
+      <c r="E111" s="0" t="n">
+        <v>2.15</v>
       </c>
       <c r="F111" s="6"/>
-      <c r="G111" s="6" t="n">
+      <c r="G111" s="0" t="n">
         <v>0.13</v>
       </c>
       <c r="H111" s="6"/>
-      <c r="I111" s="6" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="J111" s="6" t="n">
-        <v>10.89</v>
+      <c r="I111" s="0" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="J111" s="0" t="n">
+        <v>9.9</v>
       </c>
       <c r="K111" s="6"/>
       <c r="L111" s="6"/>
-      <c r="M111" s="6" t="n">
-        <v>13.29</v>
+      <c r="M111" s="0" t="n">
+        <v>12.67</v>
       </c>
       <c r="N111" s="6"/>
       <c r="O111" s="6"/>
@@ -18829,27 +18829,27 @@
       <c r="C112" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="D112" s="6" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="E112" s="6" t="n">
-        <v>2.11</v>
+      <c r="D112" s="0" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E112" s="0" t="n">
+        <v>2.24</v>
       </c>
       <c r="F112" s="6"/>
-      <c r="G112" s="6" t="n">
-        <v>0.13</v>
+      <c r="G112" s="0" t="n">
+        <v>0.12</v>
       </c>
       <c r="H112" s="6"/>
-      <c r="I112" s="6" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="J112" s="6" t="n">
-        <v>10.03</v>
+      <c r="I112" s="0" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="J112" s="0" t="n">
+        <v>10.54</v>
       </c>
       <c r="K112" s="6"/>
       <c r="L112" s="6"/>
-      <c r="M112" s="6" t="n">
-        <v>12.76</v>
+      <c r="M112" s="0" t="n">
+        <v>13.32</v>
       </c>
       <c r="N112" s="6"/>
       <c r="O112" s="6"/>
@@ -18864,27 +18864,27 @@
       <c r="C113" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="D113" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E113" s="6" t="n">
-        <v>2.85</v>
+      <c r="D113" s="0" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E113" s="0" t="n">
+        <v>2.88</v>
       </c>
       <c r="F113" s="6"/>
-      <c r="G113" s="6" t="n">
+      <c r="G113" s="0" t="n">
         <v>0.23</v>
       </c>
       <c r="H113" s="6"/>
-      <c r="I113" s="6" t="n">
-        <v>4.28</v>
-      </c>
-      <c r="J113" s="6" t="n">
-        <v>10.84</v>
+      <c r="I113" s="0" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="J113" s="0" t="n">
+        <v>10.8</v>
       </c>
       <c r="K113" s="6"/>
       <c r="L113" s="6"/>
-      <c r="M113" s="6" t="n">
-        <v>13.14</v>
+      <c r="M113" s="0" t="n">
+        <v>13.18</v>
       </c>
       <c r="N113" s="6"/>
       <c r="O113" s="6"/>
@@ -18899,27 +18899,27 @@
       <c r="C114" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="D114" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E114" s="6" t="n">
-        <v>2.87</v>
+      <c r="D114" s="0" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E114" s="0" t="n">
+        <v>2.89</v>
       </c>
       <c r="F114" s="6"/>
-      <c r="G114" s="6" t="n">
+      <c r="G114" s="0" t="n">
         <v>0.23</v>
       </c>
       <c r="H114" s="6"/>
-      <c r="I114" s="6" t="n">
-        <v>4.27</v>
-      </c>
-      <c r="J114" s="6" t="n">
-        <v>10.96</v>
+      <c r="I114" s="0" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="J114" s="0" t="n">
+        <v>10.99</v>
       </c>
       <c r="K114" s="6"/>
       <c r="L114" s="6"/>
-      <c r="M114" s="6" t="n">
-        <v>13.17</v>
+      <c r="M114" s="0" t="n">
+        <v>13.18</v>
       </c>
       <c r="N114" s="6"/>
       <c r="O114" s="6"/>
@@ -18934,27 +18934,27 @@
       <c r="C115" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="D115" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="E115" s="6" t="n">
+      <c r="D115" s="0" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E115" s="0" t="n">
         <v>2.79</v>
       </c>
       <c r="F115" s="6"/>
-      <c r="G115" s="6" t="n">
-        <v>0.24</v>
+      <c r="G115" s="0" t="n">
+        <v>0.25</v>
       </c>
       <c r="H115" s="6"/>
-      <c r="I115" s="6" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="J115" s="6" t="n">
-        <v>11.02</v>
+      <c r="I115" s="0" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="J115" s="0" t="n">
+        <v>10.92</v>
       </c>
       <c r="K115" s="6"/>
       <c r="L115" s="6"/>
-      <c r="M115" s="6" t="n">
-        <v>13.18</v>
+      <c r="M115" s="0" t="n">
+        <v>13.06</v>
       </c>
       <c r="N115" s="6"/>
       <c r="O115" s="6"/>
@@ -18969,27 +18969,27 @@
       <c r="C116" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="D116" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E116" s="6" t="n">
+      <c r="D116" s="0" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E116" s="0" t="n">
         <v>2.84</v>
       </c>
       <c r="F116" s="6"/>
-      <c r="G116" s="6" t="n">
-        <v>0.24</v>
+      <c r="G116" s="0" t="n">
+        <v>0.25</v>
       </c>
       <c r="H116" s="6"/>
-      <c r="I116" s="6" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="J116" s="6" t="n">
-        <v>11.02</v>
+      <c r="I116" s="0" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="J116" s="0" t="n">
+        <v>11.62</v>
       </c>
       <c r="K116" s="6"/>
       <c r="L116" s="6"/>
-      <c r="M116" s="6" t="n">
-        <v>13.09</v>
+      <c r="M116" s="0" t="n">
+        <v>13.06</v>
       </c>
       <c r="N116" s="6"/>
       <c r="O116" s="6"/>
@@ -19004,27 +19004,27 @@
       <c r="C117" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="D117" s="6" t="n">
+      <c r="D117" s="0" t="n">
         <v>0.57</v>
       </c>
-      <c r="E117" s="6" t="n">
-        <v>2.83</v>
+      <c r="E117" s="0" t="n">
+        <v>2.87</v>
       </c>
       <c r="F117" s="6"/>
-      <c r="G117" s="6" t="n">
+      <c r="G117" s="0" t="n">
         <v>0.25</v>
       </c>
       <c r="H117" s="6"/>
-      <c r="I117" s="6" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="J117" s="6" t="n">
-        <v>11.02</v>
+      <c r="I117" s="0" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="J117" s="0" t="n">
+        <v>11.12</v>
       </c>
       <c r="K117" s="6"/>
       <c r="L117" s="6"/>
-      <c r="M117" s="6" t="n">
-        <v>13.08</v>
+      <c r="M117" s="0" t="n">
+        <v>13.09</v>
       </c>
       <c r="N117" s="6"/>
       <c r="O117" s="6"/>
@@ -23540,7 +23540,7 @@
       <c r="D256" s="6" t="n">
         <v>9.66</v>
       </c>
-      <c r="E256" s="0" t="n">
+      <c r="E256" s="1" t="n">
         <v>0.88</v>
       </c>
       <c r="F256" s="6"/>
@@ -23550,15 +23550,15 @@
       <c r="H256" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I256" s="0" t="n">
+      <c r="I256" s="1" t="n">
         <v>0.39</v>
       </c>
       <c r="J256" s="6"/>
-      <c r="K256" s="0" t="n">
+      <c r="K256" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="L256" s="6"/>
-      <c r="M256" s="0" t="n">
+      <c r="M256" s="1" t="n">
         <v>1.71</v>
       </c>
       <c r="N256" s="6"/>
@@ -23577,25 +23577,25 @@
       <c r="D257" s="6" t="n">
         <v>9.52</v>
       </c>
-      <c r="E257" s="0" t="n">
+      <c r="E257" s="1" t="n">
         <v>0.89</v>
       </c>
       <c r="F257" s="6"/>
       <c r="G257" s="6" t="n">
         <v>7.24</v>
       </c>
-      <c r="H257" s="0" t="n">
+      <c r="H257" s="1" t="n">
         <v>0.04</v>
       </c>
-      <c r="I257" s="0" t="n">
+      <c r="I257" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="J257" s="6"/>
-      <c r="K257" s="0" t="n">
+      <c r="K257" s="1" t="n">
         <v>0.64</v>
       </c>
       <c r="L257" s="6"/>
-      <c r="M257" s="0" t="n">
+      <c r="M257" s="1" t="n">
         <v>1.88</v>
       </c>
       <c r="N257" s="6"/>
@@ -23614,25 +23614,25 @@
       <c r="D258" s="6" t="n">
         <v>9.63</v>
       </c>
-      <c r="E258" s="0" t="n">
+      <c r="E258" s="1" t="n">
         <v>0.88</v>
       </c>
       <c r="F258" s="6"/>
       <c r="G258" s="6" t="n">
         <v>6.19</v>
       </c>
-      <c r="H258" s="0" t="n">
+      <c r="H258" s="1" t="n">
         <v>0.88</v>
       </c>
-      <c r="I258" s="0" t="n">
+      <c r="I258" s="1" t="n">
         <v>0.63</v>
       </c>
       <c r="J258" s="6"/>
-      <c r="K258" s="0" t="n">
+      <c r="K258" s="1" t="n">
         <v>0.63</v>
       </c>
       <c r="L258" s="6"/>
-      <c r="M258" s="0" t="n">
+      <c r="M258" s="1" t="n">
         <v>2.84</v>
       </c>
       <c r="N258" s="6"/>
@@ -23651,25 +23651,25 @@
       <c r="D259" s="6" t="n">
         <v>8.64</v>
       </c>
-      <c r="E259" s="0" t="n">
+      <c r="E259" s="1" t="n">
         <v>0.82</v>
       </c>
       <c r="F259" s="6"/>
       <c r="G259" s="6" t="n">
         <v>1.89</v>
       </c>
-      <c r="H259" s="0" t="n">
+      <c r="H259" s="1" t="n">
         <v>3.81</v>
       </c>
-      <c r="I259" s="0" t="n">
+      <c r="I259" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="J259" s="6"/>
-      <c r="K259" s="0" t="n">
+      <c r="K259" s="1" t="n">
         <v>0.61</v>
       </c>
       <c r="L259" s="6"/>
-      <c r="M259" s="0" t="n">
+      <c r="M259" s="1" t="n">
         <v>5.06</v>
       </c>
       <c r="N259" s="6"/>
@@ -23688,25 +23688,25 @@
       <c r="D260" s="6" t="n">
         <v>1.12</v>
       </c>
-      <c r="E260" s="0" t="n">
+      <c r="E260" s="1" t="n">
         <v>0.98</v>
       </c>
       <c r="F260" s="6"/>
       <c r="G260" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="H260" s="0" t="n">
+      <c r="H260" s="1" t="n">
         <v>8.15</v>
       </c>
-      <c r="I260" s="0" t="n">
+      <c r="I260" s="1" t="n">
         <v>2.39</v>
       </c>
       <c r="J260" s="6"/>
-      <c r="K260" s="0" t="n">
+      <c r="K260" s="1" t="n">
         <v>0.58</v>
       </c>
       <c r="L260" s="6"/>
-      <c r="M260" s="0" t="n">
+      <c r="M260" s="1" t="n">
         <v>5.97</v>
       </c>
       <c r="N260" s="6"/>
@@ -23725,25 +23725,25 @@
       <c r="D261" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="E261" s="0" t="n">
+      <c r="E261" s="1" t="n">
         <v>1.11</v>
       </c>
       <c r="F261" s="6"/>
       <c r="G261" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="H261" s="0" t="n">
+      <c r="H261" s="1" t="n">
         <v>9.1</v>
       </c>
-      <c r="I261" s="0" t="n">
+      <c r="I261" s="1" t="n">
         <v>2.19</v>
       </c>
       <c r="J261" s="6"/>
-      <c r="K261" s="0" t="n">
+      <c r="K261" s="1" t="n">
         <v>0.57</v>
       </c>
       <c r="L261" s="6"/>
-      <c r="M261" s="0" t="n">
+      <c r="M261" s="1" t="n">
         <v>6.19</v>
       </c>
       <c r="N261" s="6"/>
@@ -23762,25 +23762,25 @@
       <c r="D262" s="6" t="n">
         <v>0.08</v>
       </c>
-      <c r="E262" s="0" t="n">
+      <c r="E262" s="1" t="n">
         <v>0.98</v>
       </c>
       <c r="F262" s="6"/>
       <c r="G262" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="H262" s="0" t="n">
+      <c r="H262" s="1" t="n">
         <v>9.08</v>
       </c>
-      <c r="I262" s="0" t="n">
+      <c r="I262" s="1" t="n">
         <v>2.02</v>
       </c>
       <c r="J262" s="6"/>
-      <c r="K262" s="0" t="n">
+      <c r="K262" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="L262" s="6"/>
-      <c r="M262" s="0" t="n">
+      <c r="M262" s="1" t="n">
         <v>6.42</v>
       </c>
       <c r="N262" s="6"/>
@@ -23799,25 +23799,25 @@
       <c r="D263" s="6" t="n">
         <v>0.07</v>
       </c>
-      <c r="E263" s="0" t="n">
+      <c r="E263" s="1" t="n">
         <v>0.91</v>
       </c>
       <c r="F263" s="6"/>
       <c r="G263" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="H263" s="0" t="n">
+      <c r="H263" s="1" t="n">
         <v>9.55</v>
       </c>
-      <c r="I263" s="0" t="n">
+      <c r="I263" s="1" t="n">
         <v>1.5</v>
       </c>
       <c r="J263" s="6"/>
-      <c r="K263" s="0" t="n">
+      <c r="K263" s="1" t="n">
         <v>0.54</v>
       </c>
       <c r="L263" s="6"/>
-      <c r="M263" s="0" t="n">
+      <c r="M263" s="1" t="n">
         <v>5.89</v>
       </c>
       <c r="N263" s="6"/>
@@ -23836,25 +23836,25 @@
       <c r="D264" s="6" t="n">
         <v>0.13</v>
       </c>
-      <c r="E264" s="0" t="n">
+      <c r="E264" s="1" t="n">
         <v>1.14</v>
       </c>
       <c r="F264" s="6"/>
       <c r="G264" s="6" t="n">
         <v>0.24</v>
       </c>
-      <c r="H264" s="0" t="n">
+      <c r="H264" s="1" t="n">
         <v>9.4</v>
       </c>
-      <c r="I264" s="0" t="n">
+      <c r="I264" s="1" t="n">
         <v>1.05</v>
       </c>
       <c r="J264" s="6"/>
-      <c r="K264" s="0" t="n">
+      <c r="K264" s="1" t="n">
         <v>0.63</v>
       </c>
       <c r="L264" s="6"/>
-      <c r="M264" s="0" t="n">
+      <c r="M264" s="1" t="n">
         <v>6.7</v>
       </c>
       <c r="N264" s="6"/>
@@ -23873,25 +23873,25 @@
       <c r="D265" s="6" t="n">
         <v>0.13</v>
       </c>
-      <c r="E265" s="0" t="n">
+      <c r="E265" s="1" t="n">
         <v>1.14</v>
       </c>
       <c r="F265" s="6"/>
       <c r="G265" s="6" t="n">
         <v>0.23</v>
       </c>
-      <c r="H265" s="0" t="n">
+      <c r="H265" s="1" t="n">
         <v>9.66</v>
       </c>
-      <c r="I265" s="0" t="n">
+      <c r="I265" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="J265" s="6"/>
-      <c r="K265" s="0" t="n">
+      <c r="K265" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="L265" s="6"/>
-      <c r="M265" s="0" t="n">
+      <c r="M265" s="1" t="n">
         <v>6.67</v>
       </c>
       <c r="N265" s="6"/>
@@ -23910,25 +23910,25 @@
       <c r="D266" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E266" s="0" t="n">
+      <c r="E266" s="1" t="n">
         <v>1.17</v>
       </c>
       <c r="F266" s="6"/>
       <c r="G266" s="6" t="n">
         <v>0.22</v>
       </c>
-      <c r="H266" s="0" t="n">
+      <c r="H266" s="1" t="n">
         <v>10.02</v>
       </c>
-      <c r="I266" s="0" t="n">
+      <c r="I266" s="1" t="n">
         <v>0.35</v>
       </c>
       <c r="J266" s="6"/>
-      <c r="K266" s="0" t="n">
+      <c r="K266" s="1" t="n">
         <v>0.54</v>
       </c>
       <c r="L266" s="6"/>
-      <c r="M266" s="0" t="n">
+      <c r="M266" s="1" t="n">
         <v>6.52</v>
       </c>
       <c r="N266" s="6"/>
@@ -23947,25 +23947,25 @@
       <c r="D267" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E267" s="0" t="n">
+      <c r="E267" s="1" t="n">
         <v>1.12</v>
       </c>
       <c r="F267" s="6"/>
       <c r="G267" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H267" s="0" t="n">
+      <c r="H267" s="1" t="n">
         <v>10.07</v>
       </c>
-      <c r="I267" s="0" t="n">
+      <c r="I267" s="1" t="n">
         <v>0.33</v>
       </c>
       <c r="J267" s="6"/>
-      <c r="K267" s="0" t="n">
+      <c r="K267" s="1" t="n">
         <v>0.52</v>
       </c>
       <c r="L267" s="6"/>
-      <c r="M267" s="0" t="n">
+      <c r="M267" s="1" t="n">
         <v>6.37</v>
       </c>
       <c r="N267" s="6"/>
@@ -23984,25 +23984,25 @@
       <c r="D268" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="E268" s="0" t="n">
+      <c r="E268" s="1" t="n">
         <v>1.16</v>
       </c>
       <c r="F268" s="6"/>
       <c r="G268" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H268" s="0" t="n">
+      <c r="H268" s="1" t="n">
         <v>10.39</v>
       </c>
-      <c r="I268" s="0" t="n">
+      <c r="I268" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="J268" s="6"/>
-      <c r="K268" s="0" t="n">
+      <c r="K268" s="1" t="n">
         <v>0.46</v>
       </c>
       <c r="L268" s="6"/>
-      <c r="M268" s="0" t="n">
+      <c r="M268" s="1" t="n">
         <v>6.13</v>
       </c>
       <c r="N268" s="6"/>
@@ -24021,25 +24021,25 @@
       <c r="D269" s="6" t="n">
         <v>0.11</v>
       </c>
-      <c r="E269" s="0" t="n">
+      <c r="E269" s="1" t="n">
         <v>1.17</v>
       </c>
       <c r="F269" s="6"/>
       <c r="G269" s="6" t="n">
         <v>0.21</v>
       </c>
-      <c r="H269" s="0" t="n">
+      <c r="H269" s="1" t="n">
         <v>10.55</v>
       </c>
-      <c r="I269" s="0" t="n">
+      <c r="I269" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="J269" s="6"/>
-      <c r="K269" s="0" t="n">
+      <c r="K269" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="L269" s="6"/>
-      <c r="M269" s="0" t="n">
+      <c r="M269" s="1" t="n">
         <v>6.01</v>
       </c>
       <c r="N269" s="6"/>

</xml_diff>